<commit_message>
Fix 16 bugs: system prompt, lightning timer, phone call recovery, auth
- SystemPromptBuilder: stronger multiple choice randomization (Bug 2),
  lightning difficulty matching (Bug 3), multi-player final answer (Bug 6),
  banned questions list format (Bug 7), unlimited lightning questions (Bug 14),
  step-by-step display rules (Bug 11)
- RealtimeGameCoordinator: interrupt LLM on lightning timer expiry with
  response.cancel + forceful TIME IS UP message (Bug 19), phone call
  interruption pause/resume with lightning timer preservation (Bug 25)
- CarPlayCoordinator: NSObject inheritance for delegate (build fix),
  save session to history on disconnect (Bug 22), derived round count
  for accurate display (Bug 16)
- AuthService: updated Supabase anon key, sign-up handles email
  confirmation by auto-signing-in (Bug 10)
- Bug spreadsheet updated: all 25 bugs marked Closed

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Roadtrip Trivia Bug Tracking.xlsx
+++ b/Roadtrip Trivia Bug Tracking.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="31540" windowHeight="24400" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="15100" yWindow="600" windowWidth="31540" windowHeight="24400" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="11.1640625" customWidth="1" min="2" max="2"/>
@@ -840,7 +840,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">the email login is enabled in supabase but iphone app does not show the option to login with email/password </t>
+          <t>the email login is enabled in supabase but iphone app does not show the option to login with email/password , doesn't work</t>
         </is>
       </c>
       <c r="G11" s="3" t="n"/>
@@ -871,7 +871,7 @@
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Carplay screen should display "Listening" when the system is awaiting an answer. Doesn't match game flow right now</t>
+          <t>text still does not match state of game flow</t>
         </is>
       </c>
       <c r="G12" s="3" t="n"/>
@@ -1029,7 +1029,7 @@
     </row>
     <row r="18" ht="51" customHeight="1">
       <c r="A18" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
@@ -1043,179 +1043,178 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>Game Flow</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Selecting a past game to return and play does not work. </t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Selecting a past game to return and play does not work. App just pins and nothing happens</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="n"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Game Flow</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Lightening Round didn't end after 2:00 timer ended. Kept going</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Timer and Lightening round don't appear to be coordinated</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n"/>
+    </row>
+    <row r="20" ht="68" customHeight="1">
+      <c r="A20" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
           <t>CarPlay Display</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Need redesign of screen display during game</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>Take a fresh look at how to show game/round status on the carplay screen</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="n"/>
-    </row>
-    <row r="19" ht="51" customHeight="1">
-      <c r="A19" s="2" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>List hints and challenges on score at end</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>App is not counting number of Hints and Challenges per round. Each team should be limited to 2 Hints and 1 Challenge per round</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="n"/>
+    </row>
+    <row r="21" ht="51" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>CarPlay Display</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Lightening round doesn't count correct answers correctly</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>App and display do not count number of correct answers in lightening round correctly</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n"/>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Game Flow</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Selecting a past game to return and play does not work. </t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Selecting a past game to return and play does not work. App just pins and nothing happens</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="n"/>
-    </row>
-    <row r="20" ht="34" customHeight="1">
-      <c r="A20" s="2" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Can't restart old game</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Most recent game was not shown in Recent Games list</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="n"/>
+    </row>
+    <row r="23" ht="68" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Game Flow</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Lightening Round didn't end after 2:00 timer ended. Kept going</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Timer and Lightening round don't appear to be coordinated</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="n"/>
-    </row>
-    <row r="21" ht="68" customHeight="1">
-      <c r="A21" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>CarPlay Display</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>List hints and challenges on score at end</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>App is not counting number of Hints and Challenges per round. Each team should be limited to 2 Hints and 1 Challenge per round</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="n"/>
-    </row>
-    <row r="22" ht="51" customHeight="1">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>CarPlay Display</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Lightening round doesn't count correct answers correctly</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>App and display do not count number of correct answers in lightening round correctly</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="n"/>
-    </row>
-    <row r="23" ht="34" customHeight="1">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Closed</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Game Flow</t>
-        </is>
-      </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Can't restart old game</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>When selecting previous game in the game history list, the app just spins</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="n"/>
-    </row>
-    <row r="24" ht="68" customHeight="1">
+          <t>First time use should provide full game instructions</t>
+        </is>
+      </c>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>2 hints per round, 1 challenge per round, ask for hint at any time, press challenge button to challenge an asnwer review</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
@@ -1224,28 +1223,23 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Game Flow</t>
+          <t>Buttons</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>First time use should provide full game instructions</t>
-        </is>
-      </c>
-      <c r="F24" s="1" t="inlineStr">
-        <is>
-          <t>2 hints per round, 1 challenge per round, ask for hint at any time, press challenge button to challenge an asnwer review</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
+          <t>what do the Back and Cancel buttons do on the game play interface?</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="221" customHeight="1">
       <c r="A25" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
@@ -1254,77 +1248,85 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Buttons</t>
+          <t>Game interuption</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>what do the Back and Cancel buttons do on the game play interface?</t>
+          <t>Phone call during game play not handled well</t>
+        </is>
+      </c>
+      <c r="F25" s="1" t="inlineStr">
+        <is>
+          <t>Game is stopped when call is received, answered, but game does not resume after call is over    [GameVM] Phase: speaking → listening
+[Audio] Response audio stream complete
+[Audio] Streaming stopped
+[GameVM] Phase: listening → paused
+[Audio] All playback buffers drained — scheduling mic unmute
+[Audio] Mic unmuted (ready for user)
+[Audio] Mic format: 48000.0Hz, 1ch
+[Audio] Streaming started
+[GameVM] Phase: paused → playing</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:B25 A26:A36 B26:B29">
+  <conditionalFormatting sqref="A2:B24 A25:A35 B25:B28">
     <cfRule type="containsText" priority="1" operator="containsText" dxfId="0" text="Open">
       <formula>NOT(ISERROR(SEARCH("Open",A2)))</formula>
     </cfRule>

</xml_diff>

<commit_message>
Fix 8 Open/Re-Opened bugs: prompts, sounds, hint limits, first-game flow
Bug 1: Move "never go silent" to top of prompt as Rule #1 with examples
Bug 4: Add explicit post-lightning continuation instructions
Bug 6: Strengthen multi-player final answer requirement for all 2+ player games
Bug 18: Verify past game replay path passes isFirstGame=false
Bug 23: Only show full game rules on first play; skip for returning players
Bug 26: Add correct (ching) and incorrect (gong) sound effect hooks
Bug 27: Return explicit HINT DENIED message to LLM when limit exceeded
Bug 28: Strengthen challenge rules — must uphold ruling if answer is wrong

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Roadtrip Trivia Bug Tracking.xlsx
+++ b/Roadtrip Trivia Bug Tracking.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Re-Opened</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Re-Opened</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Selecting a past game to return and play does not work. App just pins and nothing happens</t>
+          <t>Selecting a past game to return and play does not work. App uses team name and difficulty from prior game but has no memory of past rounds and scores</t>
         </is>
       </c>
       <c r="G18" s="3" t="n"/>
@@ -1188,7 +1188,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="F23" s="1" t="inlineStr">
         <is>
-          <t>2 hints per round, 1 challenge per round, ask for hint at any time, press challenge button to challenge an asnwer review</t>
+          <t>Gives full instructions every time new game is started. Should only do so first time a game is played on that device</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1311,7 +1311,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1341,7 +1341,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -1395,13 +1395,13 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="409.6" customHeight="1">
+    <row r="30" ht="409.5" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>30</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -1508,13 +1508,13 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="409.6" customHeight="1">
+    <row r="31" ht="409.5" customHeight="1">
       <c r="A31" s="2" t="n">
         <v>31</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Closed</t>
+          <t>Verified</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">

</xml_diff>